<commit_message>
use openxlsx2 instead of openxlsx and readxl
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_weighted.xlsx
+++ b/tests/testthat/excel/mapping_neu_weighted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99B06889-7736-4C0F-AE6D-6F8E7A2C8510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526D824F-5BD9-417C-93ED-4329C733A5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -209,7 +209,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="351">
   <si>
     <t>Make script</t>
   </si>
@@ -1259,6 +1259,9 @@
   </si>
   <si>
     <t>Q7</t>
+  </si>
+  <si>
+    <t>Checks</t>
   </si>
 </sst>
 </file>
@@ -6698,6 +6701,9 @@
       <c r="AN1" s="28" t="s">
         <v>257</v>
       </c>
+      <c r="AO1" s="24" t="s">
+        <v>350</v>
+      </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A2" s="19"/>

</xml_diff>